<commit_message>
Correct result tables, notes and hashes without changing any value
Grades: rename columns to strict_accuracy and answer_accuracy.
Summary: mark per-question ALR and faithfulness as not used in the paper
and add the shares of claims the paper reports. Workbook notes and the
main-flow chart title (50 questions, not 45) are corrected. Version
1000020 is marked as a repeat upload. Add retrieval_partial.jsonl named
by the manifests and .gitattributes so sealed files keep their bytes.
Remove duplicate logs.

README: gold data was written by Claude, not marked by humans. Record the
rubric difference for four partial labels and the masking that changes
two frozen hashes. No grade or metric value is changed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/research_evaluation_20261030/results/SUMMARY_TABLES.xlsx
+++ b/research_evaluation_20261030/results/SUMMARY_TABLES.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -445,21 +445,42 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Answer labels: manual reading by one author against reference answers, tuples and gold evidence (not independent).</t>
+          <t>Gold questions, reference answers, tuples and evidence regions: written by Claude from the extracted text, light text check, accepted by the project owner (frozen_20261030/gold_questions.jsonl).</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Not completed: P047-P050 (generator offline), P007 (withheld by citation check); see sheet error_cases.</t>
+          <t>Answer labels: one LLM-assisted reading pass (Claude) against reference answers, tuples and gold evidence; not independent (column grader of sheet manual_grades).</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Not used: mainflow_20261030/judgments.jsonl and report/ (automatic Qwen judge stopped after 14 of 100 answers).</t>
+          <t>Text-only main flow: all 50 answered; P047-P050 and P007 come from a second run.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Image policy: 45 of 50 answered; not completed: P047-P050 (generator offline), P007 (withheld by citation check); see sheet error_cases.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>In summary_mean_sd, *_of_claims rows are shares of all claims (used in the paper); the rows without that suffix are means over questions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Not used and not included in this repository: mainflow_20261030/judgments.jsonl and report/ (automatic Qwen judge stopped after 14 of 100 answers).</t>
         </is>
       </c>
     </row>
@@ -474,7 +495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -583,7 +604,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no (mean over questions; the paper uses the share of claims)</t>
         </is>
       </c>
     </row>
@@ -609,7 +630,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no (mean over questions; the paper uses the share of claims)</t>
         </is>
       </c>
     </row>
@@ -829,14 +850,14 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>count_correct</t>
+          <t>attribute_leakage_rate_of_claims</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>33</v>
+        <v>0.051</v>
       </c>
       <c r="E14" t="n">
-        <v>50</v>
+        <v>98</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -852,14 +873,14 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>count_partial</t>
+          <t>citation_faithfulness_of_claims</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>14</v>
+        <v>0.888</v>
       </c>
       <c r="E15" t="n">
-        <v>50</v>
+        <v>98</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -875,11 +896,11 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>count_wrong</t>
+          <t>count_correct</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>2</v>
+        <v>33</v>
       </c>
       <c r="E16" t="n">
         <v>50</v>
@@ -898,11 +919,11 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>count_no_answer</t>
+          <t>count_partial</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="E17" t="n">
         <v>50</v>
@@ -916,52 +937,46 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>image_policy</t>
+          <t>text_only</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>answer_accuracy</t>
+          <t>count_wrong</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>0.744</v>
-      </c>
-      <c r="D18" t="n">
-        <v>0.379</v>
+        <v>2</v>
       </c>
       <c r="E18" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>no (zero-shot VLM; kept for the record)</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>image_policy</t>
+          <t>text_only</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>strict_accuracy</t>
+          <t>count_no_answer</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0.644</v>
-      </c>
-      <c r="D19" t="n">
-        <v>0.484</v>
+        <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>no (zero-shot VLM; kept for the record)</t>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -973,14 +988,14 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>attribute_leakage_rate</t>
+          <t>answer_accuracy</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>0.074</v>
+        <v>0.744</v>
       </c>
       <c r="D20" t="n">
-        <v>0.206</v>
+        <v>0.379</v>
       </c>
       <c r="E20" t="n">
         <v>45</v>
@@ -999,14 +1014,14 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>citation_faithfulness</t>
+          <t>strict_accuracy</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>0.826</v>
+        <v>0.644</v>
       </c>
       <c r="D21" t="n">
-        <v>0.32</v>
+        <v>0.484</v>
       </c>
       <c r="E21" t="n">
         <v>45</v>
@@ -1025,17 +1040,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>key_value_recall</t>
+          <t>attribute_leakage_rate</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>0.775</v>
+        <v>0.074</v>
       </c>
       <c r="D22" t="n">
-        <v>0.368</v>
+        <v>0.206</v>
       </c>
       <c r="E22" t="n">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -1051,14 +1066,14 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>evidence_recall_at_10</t>
+          <t>citation_faithfulness</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>0.919</v>
+        <v>0.826</v>
       </c>
       <c r="D23" t="n">
-        <v>0.221</v>
+        <v>0.32</v>
       </c>
       <c r="E23" t="n">
         <v>45</v>
@@ -1077,17 +1092,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>evidence_precision_at_10</t>
+          <t>key_value_recall</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>0.12</v>
+        <v>0.775</v>
       </c>
       <c r="D24" t="n">
-        <v>0.055</v>
+        <v>0.368</v>
       </c>
       <c r="E24" t="n">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -1103,14 +1118,14 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>required_evidence_recall</t>
+          <t>evidence_recall_at_10</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>0.956</v>
+        <v>0.919</v>
       </c>
       <c r="D25" t="n">
-        <v>0.179</v>
+        <v>0.221</v>
       </c>
       <c r="E25" t="n">
         <v>45</v>
@@ -1129,14 +1144,14 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>citation_precision</t>
+          <t>evidence_precision_at_10</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>0.741</v>
+        <v>0.12</v>
       </c>
       <c r="D26" t="n">
-        <v>0.382</v>
+        <v>0.055</v>
       </c>
       <c r="E26" t="n">
         <v>45</v>
@@ -1155,14 +1170,14 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>citation_recall</t>
+          <t>required_evidence_recall</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>0.737</v>
+        <v>0.956</v>
       </c>
       <c r="D27" t="n">
-        <v>0.385</v>
+        <v>0.179</v>
       </c>
       <c r="E27" t="n">
         <v>45</v>
@@ -1181,18 +1196,21 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>count_correct</t>
+          <t>citation_precision</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>29</v>
+        <v>0.741</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0.382</v>
       </c>
       <c r="E28" t="n">
         <v>45</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>no (zero-shot VLM; kept for the record)</t>
         </is>
       </c>
     </row>
@@ -1204,18 +1222,21 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>count_partial</t>
+          <t>citation_recall</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>9</v>
+        <v>0.737</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0.385</v>
       </c>
       <c r="E29" t="n">
         <v>45</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>no (zero-shot VLM; kept for the record)</t>
         </is>
       </c>
     </row>
@@ -1227,14 +1248,14 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>count_wrong</t>
+          <t>attribute_leakage_rate_of_claims</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>7</v>
+        <v>0.082</v>
       </c>
       <c r="E30" t="n">
-        <v>45</v>
+        <v>85</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
@@ -1250,16 +1271,108 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
+          <t>citation_faithfulness_of_claims</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>0.835</v>
+      </c>
+      <c r="E31" t="n">
+        <v>85</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>image_policy</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>count_correct</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>29</v>
+      </c>
+      <c r="E32" t="n">
+        <v>45</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>image_policy</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>count_partial</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>9</v>
+      </c>
+      <c r="E33" t="n">
+        <v>45</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>image_policy</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>count_wrong</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>7</v>
+      </c>
+      <c r="E34" t="n">
+        <v>45</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>image_policy</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
           <t>count_no_answer</t>
         </is>
       </c>
-      <c r="C31" t="n">
+      <c r="C35" t="n">
         <v>0</v>
       </c>
-      <c r="E31" t="n">
+      <c r="E35" t="n">
         <v>45</v>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="F35" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -3977,12 +4090,12 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>accuracy</t>
+          <t>strict_accuracy</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>partial_credit</t>
+          <t>answer_accuracy</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">

</xml_diff>